<commit_message>
Chip por modelo: columna Chip en Diccionario_Modelos + motor la usa
- Estructura_PreGenerada: Diccionario_Modelos ahora trae columna Chip pre-llenada
  (detectado del nombre real; sugerido eSIM para iPhone, Dual SIM para Android)
- construirInventario usa el Chip del diccionario y, si esta vacio, lo detecta del nombre
- Asi todos los productos pueden mostrar su chip en el sitio
</commit_message>
<xml_diff>
--- a/apps-script/Estructura_PreGenerada.xlsx
+++ b/apps-script/Estructura_PreGenerada.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D299"/>
+  <dimension ref="A1:E299"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -440,6 +440,11 @@
           <t>Categoria</t>
         </is>
       </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Chip</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -462,6 +467,7 @@
           <t>Accesorios</t>
         </is>
       </c>
+      <c r="E2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -484,6 +490,7 @@
           <t>Accesorios</t>
         </is>
       </c>
+      <c r="E3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -506,6 +513,7 @@
           <t>Accesorios</t>
         </is>
       </c>
+      <c r="E4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -528,6 +536,7 @@
           <t>Accesorios</t>
         </is>
       </c>
+      <c r="E5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -550,6 +559,7 @@
           <t>Accesorios</t>
         </is>
       </c>
+      <c r="E6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -572,6 +582,7 @@
           <t>Accesorios</t>
         </is>
       </c>
+      <c r="E7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -594,6 +605,7 @@
           <t>Accesorios</t>
         </is>
       </c>
+      <c r="E8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -616,6 +628,7 @@
           <t>Accesorios</t>
         </is>
       </c>
+      <c r="E9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -638,6 +651,7 @@
           <t>Accesorios</t>
         </is>
       </c>
+      <c r="E10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -660,6 +674,7 @@
           <t>Accesorios</t>
         </is>
       </c>
+      <c r="E11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -682,6 +697,7 @@
           <t>Accesorios</t>
         </is>
       </c>
+      <c r="E12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -704,6 +720,7 @@
           <t>Accesorios</t>
         </is>
       </c>
+      <c r="E13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -726,6 +743,7 @@
           <t>Accesorios</t>
         </is>
       </c>
+      <c r="E14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -748,6 +766,7 @@
           <t>Televisores</t>
         </is>
       </c>
+      <c r="E15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -770,6 +789,7 @@
           <t>Accesorios</t>
         </is>
       </c>
+      <c r="E16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -792,6 +812,7 @@
           <t>Accesorios</t>
         </is>
       </c>
+      <c r="E17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -814,6 +835,7 @@
           <t>Consolas</t>
         </is>
       </c>
+      <c r="E18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -836,6 +858,7 @@
           <t>Televisores</t>
         </is>
       </c>
+      <c r="E19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -858,6 +881,7 @@
           <t>Relojes</t>
         </is>
       </c>
+      <c r="E20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -880,6 +904,7 @@
           <t>Relojes</t>
         </is>
       </c>
+      <c r="E21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -902,6 +927,7 @@
           <t>Relojes</t>
         </is>
       </c>
+      <c r="E22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -924,6 +950,7 @@
           <t>Relojes</t>
         </is>
       </c>
+      <c r="E23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -946,6 +973,7 @@
           <t>Accesorios</t>
         </is>
       </c>
+      <c r="E24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -968,6 +996,7 @@
           <t>Tablets</t>
         </is>
       </c>
+      <c r="E25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -990,6 +1019,7 @@
           <t>Relojes</t>
         </is>
       </c>
+      <c r="E26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1012,6 +1042,7 @@
           <t>Relojes</t>
         </is>
       </c>
+      <c r="E27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1034,6 +1065,7 @@
           <t>Relojes</t>
         </is>
       </c>
+      <c r="E28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1056,6 +1088,7 @@
           <t>Computadoras</t>
         </is>
       </c>
+      <c r="E29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1078,6 +1111,7 @@
           <t>Consolas</t>
         </is>
       </c>
+      <c r="E30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1100,6 +1134,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1122,6 +1161,7 @@
           <t>Relojes</t>
         </is>
       </c>
+      <c r="E32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1144,6 +1184,7 @@
           <t>Computadoras</t>
         </is>
       </c>
+      <c r="E33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1166,6 +1207,7 @@
           <t>Audio</t>
         </is>
       </c>
+      <c r="E34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1188,6 +1230,7 @@
           <t>Relojes</t>
         </is>
       </c>
+      <c r="E35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1210,6 +1253,7 @@
           <t>Relojes</t>
         </is>
       </c>
+      <c r="E36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1232,6 +1276,7 @@
           <t>Relojes</t>
         </is>
       </c>
+      <c r="E37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1254,6 +1299,7 @@
           <t>Tablets</t>
         </is>
       </c>
+      <c r="E38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1276,6 +1322,7 @@
           <t>Tablets</t>
         </is>
       </c>
+      <c r="E39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1298,6 +1345,7 @@
           <t>Tablets</t>
         </is>
       </c>
+      <c r="E40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1320,6 +1368,7 @@
           <t>Tablets</t>
         </is>
       </c>
+      <c r="E41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1342,6 +1391,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -1364,6 +1418,7 @@
           <t>Consolas</t>
         </is>
       </c>
+      <c r="E43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -1386,6 +1441,7 @@
           <t>Tablets</t>
         </is>
       </c>
+      <c r="E44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -1408,6 +1464,7 @@
           <t>Tablets</t>
         </is>
       </c>
+      <c r="E45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -1430,6 +1487,7 @@
           <t>Tablets</t>
         </is>
       </c>
+      <c r="E46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -1452,6 +1510,7 @@
           <t>Tablets</t>
         </is>
       </c>
+      <c r="E47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -1474,6 +1533,7 @@
           <t>Tablets</t>
         </is>
       </c>
+      <c r="E48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -1496,6 +1556,7 @@
           <t>Audio</t>
         </is>
       </c>
+      <c r="E49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -1518,6 +1579,7 @@
           <t>Relojes</t>
         </is>
       </c>
+      <c r="E50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -1540,6 +1602,7 @@
           <t>Audio</t>
         </is>
       </c>
+      <c r="E51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -1562,6 +1625,7 @@
           <t>Accesorios</t>
         </is>
       </c>
+      <c r="E52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -1584,6 +1648,7 @@
           <t>Relojes</t>
         </is>
       </c>
+      <c r="E53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -1606,6 +1671,7 @@
           <t>Tablets</t>
         </is>
       </c>
+      <c r="E54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -1628,6 +1694,7 @@
           <t>Tablets</t>
         </is>
       </c>
+      <c r="E55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -1650,6 +1717,7 @@
           <t>Relojes</t>
         </is>
       </c>
+      <c r="E56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -1672,6 +1740,7 @@
           <t>Relojes</t>
         </is>
       </c>
+      <c r="E57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -1694,6 +1763,7 @@
           <t>Relojes</t>
         </is>
       </c>
+      <c r="E58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -1716,6 +1786,7 @@
           <t>Relojes</t>
         </is>
       </c>
+      <c r="E59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -1738,6 +1809,7 @@
           <t>Relojes</t>
         </is>
       </c>
+      <c r="E60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -1760,6 +1832,7 @@
           <t>Accesorios</t>
         </is>
       </c>
+      <c r="E61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -1782,6 +1855,7 @@
           <t>Accesorios</t>
         </is>
       </c>
+      <c r="E62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -1804,6 +1878,7 @@
           <t>Accesorios</t>
         </is>
       </c>
+      <c r="E63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -1826,6 +1901,7 @@
           <t>Computadoras</t>
         </is>
       </c>
+      <c r="E64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -1848,6 +1924,7 @@
           <t>Tablets</t>
         </is>
       </c>
+      <c r="E65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -1870,6 +1947,7 @@
           <t>Consolas</t>
         </is>
       </c>
+      <c r="E66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -1892,6 +1970,7 @@
           <t>Tablets</t>
         </is>
       </c>
+      <c r="E67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -1914,6 +1993,7 @@
           <t>Relojes</t>
         </is>
       </c>
+      <c r="E68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -1936,6 +2016,7 @@
           <t>Relojes</t>
         </is>
       </c>
+      <c r="E69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -1958,6 +2039,7 @@
           <t>Relojes</t>
         </is>
       </c>
+      <c r="E70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -1980,6 +2062,7 @@
           <t>Accesorios</t>
         </is>
       </c>
+      <c r="E71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -2002,6 +2085,7 @@
           <t>Tablets</t>
         </is>
       </c>
+      <c r="E72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -2024,6 +2108,7 @@
           <t>Computadoras</t>
         </is>
       </c>
+      <c r="E73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -2046,6 +2131,7 @@
           <t>Accesorios</t>
         </is>
       </c>
+      <c r="E74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -2068,6 +2154,7 @@
           <t>Accesorios</t>
         </is>
       </c>
+      <c r="E75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -2090,6 +2177,7 @@
           <t>Accesorios</t>
         </is>
       </c>
+      <c r="E76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -2112,6 +2200,7 @@
           <t>Accesorios</t>
         </is>
       </c>
+      <c r="E77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -2134,6 +2223,7 @@
           <t>Tablets</t>
         </is>
       </c>
+      <c r="E78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -2156,6 +2246,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -2178,6 +2273,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>1 SIM</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -2200,6 +2300,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -2222,6 +2327,7 @@
           <t>Tablets</t>
         </is>
       </c>
+      <c r="E82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -2244,6 +2350,7 @@
           <t>Accesorios</t>
         </is>
       </c>
+      <c r="E83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -2266,6 +2373,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -2288,6 +2400,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -2310,6 +2427,7 @@
           <t>Tablets</t>
         </is>
       </c>
+      <c r="E86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -2332,6 +2450,7 @@
           <t>Consolas</t>
         </is>
       </c>
+      <c r="E87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -2354,6 +2473,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -2376,6 +2500,7 @@
           <t>Tablets</t>
         </is>
       </c>
+      <c r="E89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -2398,6 +2523,7 @@
           <t>Tablets</t>
         </is>
       </c>
+      <c r="E90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -2420,6 +2546,7 @@
           <t>Tablets</t>
         </is>
       </c>
+      <c r="E91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -2442,6 +2569,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -2464,6 +2596,7 @@
           <t>Computadoras</t>
         </is>
       </c>
+      <c r="E93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -2486,6 +2619,7 @@
           <t>Computadoras</t>
         </is>
       </c>
+      <c r="E94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -2508,6 +2642,7 @@
           <t>Tablets</t>
         </is>
       </c>
+      <c r="E95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -2530,6 +2665,7 @@
           <t>Computadoras</t>
         </is>
       </c>
+      <c r="E96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -2552,6 +2688,7 @@
           <t>Tablets</t>
         </is>
       </c>
+      <c r="E97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -2574,6 +2711,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -2596,6 +2738,7 @@
           <t>Tablets</t>
         </is>
       </c>
+      <c r="E99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -2618,6 +2761,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>eSIM</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -2640,6 +2788,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>eSIM</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -2662,6 +2815,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>eSIM</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -2684,6 +2842,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>eSIM</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -2706,6 +2869,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>eSIM</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -2728,6 +2896,7 @@
           <t>Tablets</t>
         </is>
       </c>
+      <c r="E105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -2750,6 +2919,7 @@
           <t>Tablets</t>
         </is>
       </c>
+      <c r="E106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -2772,6 +2942,7 @@
           <t>Computadoras</t>
         </is>
       </c>
+      <c r="E107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -2794,6 +2965,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -2816,6 +2992,7 @@
           <t>Consolas</t>
         </is>
       </c>
+      <c r="E109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -2838,6 +3015,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -2860,6 +3042,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -2882,6 +3069,7 @@
           <t>Tablets</t>
         </is>
       </c>
+      <c r="E112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -2904,6 +3092,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>eSIM</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -2926,6 +3119,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>eSIM</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -2948,6 +3146,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>eSIM</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -2970,6 +3173,7 @@
           <t>Audio</t>
         </is>
       </c>
+      <c r="E116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -2992,6 +3196,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -3014,6 +3223,7 @@
           <t>Tablets</t>
         </is>
       </c>
+      <c r="E118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -3036,6 +3246,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -3058,6 +3273,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -3080,6 +3300,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -3102,6 +3327,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -3124,6 +3354,7 @@
           <t>Tablets</t>
         </is>
       </c>
+      <c r="E123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -3146,6 +3377,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -3168,6 +3404,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -3190,6 +3431,7 @@
           <t>Accesorios</t>
         </is>
       </c>
+      <c r="E126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -3212,6 +3454,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -3234,6 +3481,7 @@
           <t>Tablets</t>
         </is>
       </c>
+      <c r="E128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -3256,6 +3504,7 @@
           <t>Relojes</t>
         </is>
       </c>
+      <c r="E129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -3278,6 +3527,7 @@
           <t>Relojes</t>
         </is>
       </c>
+      <c r="E130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -3300,6 +3550,7 @@
           <t>Relojes</t>
         </is>
       </c>
+      <c r="E131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -3322,6 +3573,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>eSIM</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -3344,6 +3600,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>eSIM</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -3366,6 +3627,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>eSIM</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -3388,6 +3654,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -3410,6 +3681,7 @@
           <t>Accesorios</t>
         </is>
       </c>
+      <c r="E136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -3432,6 +3704,7 @@
           <t>Accesorios</t>
         </is>
       </c>
+      <c r="E137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -3454,6 +3727,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -3476,6 +3754,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -3498,6 +3781,7 @@
           <t>Accesorios</t>
         </is>
       </c>
+      <c r="E140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -3520,6 +3804,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -3542,6 +3831,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -3564,6 +3858,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -3586,6 +3885,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -3608,6 +3912,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -3630,6 +3939,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -3652,6 +3966,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -3674,6 +3993,7 @@
           <t>Consolas</t>
         </is>
       </c>
+      <c r="E148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -3696,6 +4016,7 @@
           <t>Tablets</t>
         </is>
       </c>
+      <c r="E149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -3718,6 +4039,7 @@
           <t>Tablets</t>
         </is>
       </c>
+      <c r="E150" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -3740,6 +4062,7 @@
           <t>Tablets</t>
         </is>
       </c>
+      <c r="E151" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -3762,6 +4085,7 @@
           <t>Tablets</t>
         </is>
       </c>
+      <c r="E152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -3784,6 +4108,7 @@
           <t>Relojes</t>
         </is>
       </c>
+      <c r="E153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -3806,6 +4131,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -3828,6 +4158,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>eSIM</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -3850,6 +4185,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>eSIM</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -3872,6 +4212,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>eSIM</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -3894,6 +4239,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>eSIM</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -3916,6 +4266,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>eSIM</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -3938,6 +4293,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>eSIM</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -3960,6 +4320,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>eSIM</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -3982,6 +4347,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>eSIM</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -4004,6 +4374,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>eSIM</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -4026,6 +4401,7 @@
           <t>Audio</t>
         </is>
       </c>
+      <c r="E164" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -4048,6 +4424,7 @@
           <t>Audio</t>
         </is>
       </c>
+      <c r="E165" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -4070,6 +4447,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -4092,6 +4474,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -4114,6 +4501,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -4136,6 +4528,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -4158,6 +4555,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -4180,6 +4582,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -4202,6 +4609,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -4224,6 +4636,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -4246,6 +4663,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -4268,6 +4690,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>1 SIM</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -4290,6 +4717,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>1 SIM</t>
+        </is>
+      </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -4312,6 +4744,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>eSIM</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -4334,6 +4771,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -4356,6 +4798,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -4378,6 +4825,7 @@
           <t>Tablets</t>
         </is>
       </c>
+      <c r="E180" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -4400,6 +4848,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>eSIM</t>
+        </is>
+      </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -4422,6 +4875,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>eSIM</t>
+        </is>
+      </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -4444,6 +4902,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>eSIM</t>
+        </is>
+      </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -4466,6 +4929,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>eSIM</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -4488,6 +4956,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>eSIM</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -4510,6 +4983,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>eSIM</t>
+        </is>
+      </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -4532,6 +5010,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>eSIM</t>
+        </is>
+      </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -4554,6 +5037,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -4576,6 +5064,7 @@
           <t>Audio</t>
         </is>
       </c>
+      <c r="E189" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -4598,6 +5087,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -4620,6 +5114,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -4642,6 +5141,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -4664,6 +5168,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -4686,6 +5195,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -4708,6 +5222,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -4730,6 +5249,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -4752,6 +5276,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -4774,6 +5303,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -4796,6 +5330,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -4818,6 +5357,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -4840,6 +5384,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>1 SIM</t>
+        </is>
+      </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -4862,6 +5411,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>1 SIM</t>
+        </is>
+      </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
@@ -4884,6 +5438,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
@@ -4906,6 +5465,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
@@ -4928,6 +5492,7 @@
           <t>Tablets</t>
         </is>
       </c>
+      <c r="E205" t="inlineStr"/>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
@@ -4950,6 +5515,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
@@ -4972,6 +5542,7 @@
           <t>Accesorios</t>
         </is>
       </c>
+      <c r="E207" t="inlineStr"/>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
@@ -4994,6 +5565,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
@@ -5016,6 +5592,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
@@ -5038,6 +5619,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
@@ -5060,6 +5646,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
@@ -5082,6 +5673,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
@@ -5104,6 +5700,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
@@ -5126,6 +5727,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
@@ -5148,6 +5754,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
@@ -5170,6 +5781,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
@@ -5192,6 +5808,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
@@ -5214,6 +5835,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
@@ -5236,6 +5862,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
@@ -5258,6 +5889,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
@@ -5280,6 +5916,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>1 SIM</t>
+        </is>
+      </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
@@ -5302,6 +5943,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
@@ -5324,6 +5970,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
@@ -5346,6 +5997,7 @@
           <t>Consolas</t>
         </is>
       </c>
+      <c r="E224" t="inlineStr"/>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
@@ -5368,6 +6020,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
@@ -5390,6 +6047,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
@@ -5412,6 +6074,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
@@ -5434,6 +6101,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>eSIM</t>
+        </is>
+      </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
@@ -5456,6 +6128,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>eSIM</t>
+        </is>
+      </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
@@ -5478,6 +6155,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>eSIM</t>
+        </is>
+      </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
@@ -5500,6 +6182,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>eSIM</t>
+        </is>
+      </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
@@ -5522,6 +6209,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>eSIM</t>
+        </is>
+      </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
@@ -5544,6 +6236,7 @@
           <t>Audio</t>
         </is>
       </c>
+      <c r="E233" t="inlineStr"/>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
@@ -5566,6 +6259,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
@@ -5588,6 +6286,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
@@ -5610,6 +6313,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
@@ -5632,6 +6340,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
@@ -5654,6 +6367,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
@@ -5676,6 +6394,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
@@ -5698,6 +6421,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
@@ -5720,6 +6448,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
@@ -5742,6 +6475,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>eSIM</t>
+        </is>
+      </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
@@ -5764,6 +6502,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>eSIM</t>
+        </is>
+      </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
@@ -5786,6 +6529,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>eSIM</t>
+        </is>
+      </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
@@ -5808,6 +6556,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>eSIM</t>
+        </is>
+      </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
@@ -5830,6 +6583,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>eSIM</t>
+        </is>
+      </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
@@ -5852,6 +6610,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>eSIM</t>
+        </is>
+      </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
@@ -5874,6 +6637,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>eSIM</t>
+        </is>
+      </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
@@ -5896,6 +6664,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E249" t="inlineStr">
+        <is>
+          <t>eSIM</t>
+        </is>
+      </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
@@ -5918,6 +6691,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
@@ -5940,6 +6718,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
@@ -5962,6 +6745,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
@@ -5984,6 +6772,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
@@ -6006,6 +6799,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
@@ -6028,6 +6826,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
@@ -6050,6 +6853,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
@@ -6072,6 +6880,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
@@ -6094,6 +6907,7 @@
           <t>Audio</t>
         </is>
       </c>
+      <c r="E258" t="inlineStr"/>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
@@ -6116,6 +6930,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
@@ -6138,6 +6957,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
@@ -6160,6 +6984,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
@@ -6182,6 +7011,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
@@ -6204,6 +7038,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
@@ -6226,6 +7065,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E264" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
@@ -6248,6 +7092,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>1 SIM</t>
+        </is>
+      </c>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
@@ -6270,6 +7119,7 @@
           <t>Tablets</t>
         </is>
       </c>
+      <c r="E266" t="inlineStr"/>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
@@ -6292,6 +7142,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>eSIM</t>
+        </is>
+      </c>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
@@ -6314,6 +7169,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>eSIM</t>
+        </is>
+      </c>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
@@ -6336,6 +7196,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
@@ -6358,6 +7223,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
@@ -6380,6 +7250,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
@@ -6402,6 +7277,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E272" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
@@ -6424,6 +7304,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>eSIM</t>
+        </is>
+      </c>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
@@ -6446,6 +7331,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
@@ -6468,6 +7358,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
@@ -6490,6 +7385,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E276" t="inlineStr">
+        <is>
+          <t>eSIM</t>
+        </is>
+      </c>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
@@ -6512,6 +7412,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E277" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
@@ -6534,6 +7439,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E278" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
@@ -6556,6 +7466,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
@@ -6578,6 +7493,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
@@ -6600,6 +7520,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E281" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="282">
       <c r="A282" t="inlineStr">
@@ -6622,6 +7547,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E282" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
@@ -6644,6 +7574,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E283" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
@@ -6666,6 +7601,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E284" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
@@ -6688,6 +7628,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
@@ -6710,6 +7655,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="287">
       <c r="A287" t="inlineStr">
@@ -6732,6 +7682,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="288">
       <c r="A288" t="inlineStr">
@@ -6754,6 +7709,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="289">
       <c r="A289" t="inlineStr">
@@ -6776,6 +7736,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E289" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="290">
       <c r="A290" t="inlineStr">
@@ -6798,6 +7763,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E290" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="291">
       <c r="A291" t="inlineStr">
@@ -6820,6 +7790,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="292">
       <c r="A292" t="inlineStr">
@@ -6842,6 +7817,7 @@
           <t>Accesorios</t>
         </is>
       </c>
+      <c r="E292" t="inlineStr"/>
     </row>
     <row r="293">
       <c r="A293" t="inlineStr">
@@ -6864,6 +7840,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="294">
       <c r="A294" t="inlineStr">
@@ -6886,6 +7867,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
@@ -6908,6 +7894,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="296">
       <c r="A296" t="inlineStr">
@@ -6930,6 +7921,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="297">
       <c r="A297" t="inlineStr">
@@ -6952,6 +7948,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="298">
       <c r="A298" t="inlineStr">
@@ -6974,6 +7975,11 @@
           <t>Celulares</t>
         </is>
       </c>
+      <c r="E298" t="inlineStr">
+        <is>
+          <t>Dual SIM</t>
+        </is>
+      </c>
     </row>
     <row r="299">
       <c r="A299" t="inlineStr">
@@ -6994,6 +8000,11 @@
       <c r="D299" t="inlineStr">
         <is>
           <t>Celulares</t>
+        </is>
+      </c>
+      <c r="E299" t="inlineStr">
+        <is>
+          <t>eSIM</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Unificar chip: SIM suelto (iPhone) ahora es 1 SIM, consistente con Samsung
</commit_message>
<xml_diff>
--- a/apps-script/Estructura_PreGenerada.xlsx
+++ b/apps-script/Estructura_PreGenerada.xlsx
@@ -3139,7 +3139,7 @@
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>1 SIM</t>
         </is>
       </c>
     </row>
@@ -3193,7 +3193,7 @@
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>1 SIM</t>
         </is>
       </c>
     </row>
@@ -3247,7 +3247,7 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>1 SIM</t>
         </is>
       </c>
     </row>
@@ -3301,7 +3301,7 @@
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>1 SIM</t>
         </is>
       </c>
     </row>
@@ -3578,7 +3578,7 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>1 SIM</t>
         </is>
       </c>
     </row>
@@ -3605,7 +3605,7 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>1 SIM</t>
         </is>
       </c>
     </row>
@@ -3632,7 +3632,7 @@
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>1 SIM</t>
         </is>
       </c>
     </row>
@@ -4167,7 +4167,7 @@
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>1 SIM</t>
         </is>
       </c>
     </row>
@@ -4221,7 +4221,7 @@
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>1 SIM</t>
         </is>
       </c>
     </row>
@@ -4302,7 +4302,7 @@
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>1 SIM</t>
         </is>
       </c>
     </row>
@@ -5076,7 +5076,7 @@
       </c>
       <c r="E188" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>1 SIM</t>
         </is>
       </c>
     </row>
@@ -5103,7 +5103,7 @@
       </c>
       <c r="E189" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>1 SIM</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Revertir: mantener SIM (iPhone) y 1 SIM (Samsung) como chips distintos
</commit_message>
<xml_diff>
--- a/apps-script/Estructura_PreGenerada.xlsx
+++ b/apps-script/Estructura_PreGenerada.xlsx
@@ -3139,7 +3139,7 @@
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>1 SIM</t>
+          <t>SIM</t>
         </is>
       </c>
     </row>
@@ -3193,7 +3193,7 @@
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>1 SIM</t>
+          <t>SIM</t>
         </is>
       </c>
     </row>
@@ -3247,7 +3247,7 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>1 SIM</t>
+          <t>SIM</t>
         </is>
       </c>
     </row>
@@ -3301,7 +3301,7 @@
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>1 SIM</t>
+          <t>SIM</t>
         </is>
       </c>
     </row>
@@ -3578,7 +3578,7 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>1 SIM</t>
+          <t>SIM</t>
         </is>
       </c>
     </row>
@@ -3605,7 +3605,7 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>1 SIM</t>
+          <t>SIM</t>
         </is>
       </c>
     </row>
@@ -3632,7 +3632,7 @@
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>1 SIM</t>
+          <t>SIM</t>
         </is>
       </c>
     </row>
@@ -4167,7 +4167,7 @@
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>1 SIM</t>
+          <t>SIM</t>
         </is>
       </c>
     </row>
@@ -4221,7 +4221,7 @@
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>1 SIM</t>
+          <t>SIM</t>
         </is>
       </c>
     </row>
@@ -4302,7 +4302,7 @@
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>1 SIM</t>
+          <t>SIM</t>
         </is>
       </c>
     </row>
@@ -5076,7 +5076,7 @@
       </c>
       <c r="E188" t="inlineStr">
         <is>
-          <t>1 SIM</t>
+          <t>SIM</t>
         </is>
       </c>
     </row>
@@ -5103,7 +5103,7 @@
       </c>
       <c r="E189" t="inlineStr">
         <is>
-          <t>1 SIM</t>
+          <t>SIM</t>
         </is>
       </c>
     </row>

</xml_diff>